<commit_message>
Sync fee records for 2026-2027
Updated the first-term student fee data to reflect a payment of 43,000 for ADEDOJA FAITH MORAYOOLUWA, reducing the outstanding balance to 1,280. Also refreshed the related Excel sources (2026 - 2027 FEE.xlsx and parent_codes.xlsx) so the exported records stay aligned with the current student payment data.
</commit_message>
<xml_diff>
--- a/2026 - 2027 FEE.xlsx
+++ b/2026 - 2027 FEE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A16758B-C668-4C10-8774-B70E2515AE17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{056D1BA0-9702-4A36-843B-44663388CA0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="256">
   <si>
     <t>LAST NAME</t>
   </si>
@@ -800,6 +800,12 @@
   <si>
     <t>CRECHE</t>
   </si>
+  <si>
+    <t>NIP:PAUL SUNDAY ADEDOJA</t>
+  </si>
+  <si>
+    <t>ADEDOJA FAMILY</t>
+  </si>
 </sst>
 </file>
 
@@ -8750,11 +8756,11 @@
         <v>44280</v>
       </c>
       <c r="AA71" s="24">
-        <v>0</v>
+        <v>43000</v>
       </c>
       <c r="AB71" s="20">
         <f>Z71-AA71</f>
-        <v>44280</v>
+        <v>1280</v>
       </c>
       <c r="AC71" s="24" t="str">
         <f>IF(AND($T71=6000, ($T71+$W71-$AB71)&gt;=6000),T71,"")</f>
@@ -13949,11 +13955,11 @@
       </c>
       <c r="AA121" s="27">
         <f>SUM(AA2:AA120)</f>
-        <v>48000</v>
+        <v>91000</v>
       </c>
       <c r="AB121" s="27">
         <f>SUM(AB2:AB120)</f>
-        <v>7203495</v>
+        <v>7160495</v>
       </c>
       <c r="AC121" s="27">
         <f>SUM(AC2:AC120)</f>
@@ -22239,7 +22245,23 @@
         <v>252</v>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>46255</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="D3" s="9">
+        <v>43000</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>255</v>
+      </c>
+    </row>
     <row r="4" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>